<commit_message>
next stages and audits
</commit_message>
<xml_diff>
--- a/outputs/04_individual_models/csf_feature_selection.xlsx
+++ b/outputs/04_individual_models/csf_feature_selection.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="145" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="145" uniqueCount="49">
   <si>
     <t>field</t>
   </si>
@@ -63,7 +63,7 @@
     <t>note</t>
   </si>
   <si>
-    <t>CSF only</t>
+    <t>CSF</t>
   </si>
   <si>
     <t>&gt;= 50%</t>
@@ -115,9 +115,6 @@
   </si>
   <si>
     <t>ELE_censored_ptau</t>
-  </si>
-  <si>
-    <t>CSF</t>
   </si>
   <si>
     <t>analyte</t>
@@ -683,13 +680,13 @@
         <v>27</v>
       </c>
       <c r="C2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D2" t="s">
         <v>32</v>
       </c>
-      <c r="D2" t="s">
-        <v>33</v>
-      </c>
       <c r="E2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="F2">
         <v>-1.276599</v>
@@ -698,7 +695,7 @@
         <v>1.276599</v>
       </c>
       <c r="H2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="I2">
         <v>1</v>
@@ -715,13 +712,13 @@
         <v>28</v>
       </c>
       <c r="C3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D3" t="s">
         <v>32</v>
       </c>
-      <c r="D3" t="s">
-        <v>33</v>
-      </c>
       <c r="E3" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="F3">
         <v>0.581348</v>
@@ -730,7 +727,7 @@
         <v>0.581348</v>
       </c>
       <c r="H3" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="I3">
         <v>1</v>
@@ -747,13 +744,13 @@
         <v>29</v>
       </c>
       <c r="C4" t="s">
-        <v>32</v>
+        <v>14</v>
       </c>
       <c r="D4" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E4" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="F4">
         <v>0.397857</v>
@@ -762,7 +759,7 @@
         <v>0.397857</v>
       </c>
       <c r="H4" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="I4">
         <v>1</v>
@@ -779,13 +776,13 @@
         <v>30</v>
       </c>
       <c r="C5" t="s">
-        <v>32</v>
+        <v>14</v>
       </c>
       <c r="D5" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E5" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="F5">
         <v>-0.07373300000000001</v>
@@ -794,7 +791,7 @@
         <v>0.07373300000000001</v>
       </c>
       <c r="H5" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="I5">
         <v>1</v>
@@ -811,13 +808,13 @@
         <v>31</v>
       </c>
       <c r="C6" t="s">
-        <v>32</v>
+        <v>14</v>
       </c>
       <c r="D6" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E6" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="F6">
         <v>-0.03954</v>
@@ -826,7 +823,7 @@
         <v>0.03954</v>
       </c>
       <c r="H6" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="I6">
         <v>1</v>
@@ -864,16 +861,16 @@
     </row>
     <row r="2" spans="1:5">
       <c r="A2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C2" t="s">
         <v>32</v>
       </c>
-      <c r="C2" t="s">
-        <v>33</v>
-      </c>
       <c r="D2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E2">
         <v>99.59999999999999</v>
@@ -881,16 +878,16 @@
     </row>
     <row r="3" spans="1:5">
       <c r="A3" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B3" t="s">
-        <v>32</v>
+        <v>14</v>
       </c>
       <c r="C3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D3" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E3">
         <v>100</v>
@@ -898,16 +895,16 @@
     </row>
     <row r="4" spans="1:5">
       <c r="A4" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B4" t="s">
-        <v>32</v>
+        <v>14</v>
       </c>
       <c r="C4" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D4" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E4">
         <v>100</v>
@@ -915,16 +912,16 @@
     </row>
     <row r="5" spans="1:5">
       <c r="A5" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B5" t="s">
-        <v>32</v>
+        <v>14</v>
       </c>
       <c r="C5" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D5" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E5">
         <v>99.7</v>
@@ -945,21 +942,21 @@
         <v>19</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>47</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>48</v>
       </c>
     </row>
     <row r="2" spans="1:5">
       <c r="A2" t="s">
-        <v>32</v>
+        <v>14</v>
       </c>
       <c r="B2">
         <v>9</v>
@@ -992,24 +989,24 @@
         <v>20</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>47</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>48</v>
       </c>
     </row>
     <row r="2" spans="1:6">
       <c r="A2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B2" t="s">
         <v>32</v>
-      </c>
-      <c r="B2" t="s">
-        <v>33</v>
       </c>
       <c r="C2">
         <v>3</v>
@@ -1026,10 +1023,10 @@
     </row>
     <row r="3" spans="1:6">
       <c r="A3" t="s">
-        <v>32</v>
+        <v>14</v>
       </c>
       <c r="B3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C3">
         <v>4</v>
@@ -1046,10 +1043,10 @@
     </row>
     <row r="4" spans="1:6">
       <c r="A4" t="s">
-        <v>32</v>
+        <v>14</v>
       </c>
       <c r="B4" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C4">
         <v>2</v>
@@ -1108,13 +1105,13 @@
         <v>27</v>
       </c>
       <c r="B2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C2" t="s">
         <v>32</v>
       </c>
-      <c r="C2" t="s">
-        <v>33</v>
-      </c>
       <c r="D2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E2">
         <v>-1.276599</v>
@@ -1123,7 +1120,7 @@
         <v>1.276599</v>
       </c>
       <c r="G2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="H2">
         <v>1</v>
@@ -1137,13 +1134,13 @@
         <v>28</v>
       </c>
       <c r="B3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C3" t="s">
         <v>32</v>
       </c>
-      <c r="C3" t="s">
-        <v>33</v>
-      </c>
       <c r="D3" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E3">
         <v>0.581348</v>
@@ -1152,7 +1149,7 @@
         <v>0.581348</v>
       </c>
       <c r="G3" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="H3">
         <v>1</v>
@@ -1166,13 +1163,13 @@
         <v>29</v>
       </c>
       <c r="B4" t="s">
-        <v>32</v>
+        <v>14</v>
       </c>
       <c r="C4" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D4" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E4">
         <v>0.397857</v>
@@ -1181,7 +1178,7 @@
         <v>0.397857</v>
       </c>
       <c r="G4" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="H4">
         <v>1</v>
@@ -1195,13 +1192,13 @@
         <v>30</v>
       </c>
       <c r="B5" t="s">
-        <v>32</v>
+        <v>14</v>
       </c>
       <c r="C5" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D5" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E5">
         <v>-0.07373300000000001</v>
@@ -1210,7 +1207,7 @@
         <v>0.07373300000000001</v>
       </c>
       <c r="G5" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="H5">
         <v>1</v>
@@ -1224,13 +1221,13 @@
         <v>31</v>
       </c>
       <c r="B6" t="s">
-        <v>32</v>
+        <v>14</v>
       </c>
       <c r="C6" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D6" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E6">
         <v>-0.03954</v>
@@ -1239,7 +1236,7 @@
         <v>0.03954</v>
       </c>
       <c r="G6" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="H6">
         <v>1</v>
@@ -1250,16 +1247,16 @@
     </row>
     <row r="7" spans="1:9">
       <c r="A7" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B7" t="s">
-        <v>32</v>
+        <v>14</v>
       </c>
       <c r="C7" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D7" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E7">
         <v>0</v>
@@ -1268,7 +1265,7 @@
         <v>0</v>
       </c>
       <c r="G7" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="H7">
         <v>0</v>
@@ -1279,16 +1276,16 @@
     </row>
     <row r="8" spans="1:9">
       <c r="A8" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B8" t="s">
-        <v>32</v>
+        <v>14</v>
       </c>
       <c r="C8" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D8" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E8">
         <v>0</v>
@@ -1297,7 +1294,7 @@
         <v>0</v>
       </c>
       <c r="G8" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="H8">
         <v>0</v>
@@ -1308,16 +1305,16 @@
     </row>
     <row r="9" spans="1:9">
       <c r="A9" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B9" t="s">
+        <v>14</v>
+      </c>
+      <c r="C9" t="s">
         <v>32</v>
       </c>
-      <c r="C9" t="s">
-        <v>33</v>
-      </c>
       <c r="D9" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E9">
         <v>0</v>
@@ -1326,7 +1323,7 @@
         <v>0</v>
       </c>
       <c r="G9" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="H9">
         <v>0</v>
@@ -1337,16 +1334,16 @@
     </row>
     <row r="10" spans="1:9">
       <c r="A10" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B10" t="s">
-        <v>32</v>
+        <v>14</v>
       </c>
       <c r="C10" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D10" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E10">
         <v>0</v>
@@ -1355,7 +1352,7 @@
         <v>0</v>
       </c>
       <c r="G10" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="H10">
         <v>0</v>

</xml_diff>